<commit_message>
Adiciona imagens do logo e lupa
</commit_message>
<xml_diff>
--- a/dados/excel/distribuicao_salarial.xlsx
+++ b/dados/excel/distribuicao_salarial.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Série temporal" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dados'!$A$1:$K$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dados'!$A$1:$K$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10">
@@ -628,7 +628,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026 19:18</t>
+          <t>10/10/2026 14:55</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2891,8 +2891,43 @@
         <v>34321.4</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B58" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="C58" s="9" t="n">
+        <v>14368</v>
+      </c>
+      <c r="D58" s="10" t="n">
+        <v>8441.040000000001</v>
+      </c>
+      <c r="E58" s="10" t="n">
+        <v>1864</v>
+      </c>
+      <c r="F58" s="10" t="n">
+        <v>3725.13</v>
+      </c>
+      <c r="G58" s="10" t="n">
+        <v>6154.53</v>
+      </c>
+      <c r="H58" s="10" t="n">
+        <v>11948.15</v>
+      </c>
+      <c r="I58" s="10" t="n">
+        <v>16886.77</v>
+      </c>
+      <c r="J58" s="10" t="n">
+        <v>21572.64</v>
+      </c>
+      <c r="K58" s="10" t="n">
+        <v>34412.59</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K57"/>
+  <autoFilter ref="A1:K58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>